<commit_message>
Experiment Log Update + Exported Google Sheets
</commit_message>
<xml_diff>
--- a/reports/sheets/Sorter_Model_Sweep_Results.xlsx
+++ b/reports/sheets/Sorter_Model_Sweep_Results.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eval Results'!$A$1:$DK$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eval Results'!$A$1:$DK$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DK7"/>
+  <dimension ref="A1:DK9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2971,8 +2971,724 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>deepseek-v4-pro_sorter_v13_subtype_langfuse</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>509</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Pro</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>v13</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.9961</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.9528</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>0.9548</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>0.9555</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>509</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>0.9332</v>
+      </c>
+      <c r="N8" s="6" t="n">
+        <v>0.9705</v>
+      </c>
+      <c r="O8" s="6" t="n">
+        <v>0.0186</v>
+      </c>
+      <c r="P8" s="6" t="n">
+        <v>0.9902</v>
+      </c>
+      <c r="Q8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>0.0049</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="X8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="6" t="n">
+        <v>0.9231</v>
+      </c>
+      <c r="Z8" s="6" t="n">
+        <v>0.9545</v>
+      </c>
+      <c r="AA8" s="6" t="n">
+        <v>0.8846000000000001</v>
+      </c>
+      <c r="AB8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC8" s="6" t="n">
+        <v>0.9286</v>
+      </c>
+      <c r="AD8" s="6" t="n">
+        <v>0.9688</v>
+      </c>
+      <c r="AE8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF8" s="6" t="n">
+        <v>0.8667</v>
+      </c>
+      <c r="AG8" s="6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AH8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ8" s="6" t="n">
+        <v>0.9091</v>
+      </c>
+      <c r="AK8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM8" s="6" t="n">
+        <v>0.8824</v>
+      </c>
+      <c r="AN8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO8" s="6" t="n">
+        <v>0.9444</v>
+      </c>
+      <c r="AP8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR8" s="6" t="n">
+        <v>0.8214</v>
+      </c>
+      <c r="AS8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU8" s="6" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="AV8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX8" s="6" t="n">
+        <v>0.9231</v>
+      </c>
+      <c r="AY8" s="6" t="n">
+        <v>0.9545</v>
+      </c>
+      <c r="AZ8" s="6" t="n">
+        <v>0.8846000000000001</v>
+      </c>
+      <c r="BA8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB8" s="6" t="n">
+        <v>0.9286</v>
+      </c>
+      <c r="BC8" s="6" t="n">
+        <v>0.9688</v>
+      </c>
+      <c r="BD8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE8" s="6" t="n">
+        <v>0.8667</v>
+      </c>
+      <c r="BF8" s="6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="BG8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI8" s="6" t="n">
+        <v>0.9394</v>
+      </c>
+      <c r="BJ8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL8" s="6" t="n">
+        <v>0.8824</v>
+      </c>
+      <c r="BM8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN8" s="6" t="n">
+        <v>0.9444</v>
+      </c>
+      <c r="BO8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ8" s="6" t="n">
+        <v>0.8214</v>
+      </c>
+      <c r="BR8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT8" s="6" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="BU8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="BW8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="BX8" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="BY8" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="BZ8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="CA8" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="CB8" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="CC8" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="CD8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="CE8" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="CF8" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="CG8" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="CH8" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="CI8" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="CJ8" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="CK8" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="CL8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CM8" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="CN8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="CO8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="CP8" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="CQ8" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="CR8" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="CS8" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="CT8" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="CU8" s="4" t="n">
+        <v>6696462</v>
+      </c>
+      <c r="CV8" s="4" t="n">
+        <v>274110</v>
+      </c>
+      <c r="CW8" s="4" t="n">
+        <v>6970572</v>
+      </c>
+      <c r="CX8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ8" s="5" t="n">
+        <v>3.151437</v>
+      </c>
+      <c r="DA8" s="4" t="n">
+        <v>509</v>
+      </c>
+      <c r="DB8" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DC8" s="4" t="n">
+        <v>4096</v>
+      </c>
+      <c r="DD8" s="4" t="n">
+        <v>100000</v>
+      </c>
+      <c r="DE8" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="DF8" s="3" t="inlineStr">
+        <is>
+          <t>llm-mailroom/mailroom-cuad-contracts-full</t>
+        </is>
+      </c>
+      <c r="DG8" s="4" t="n">
+        <v>509</v>
+      </c>
+      <c r="DH8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="DI8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ8" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="DK8" s="3" t="inlineStr">
+        <is>
+          <t>Full-509 benchmark (KANBAN-042) — deepseek v4 PRO arm ($0.435/M prompt + $0.87/M completion; ~$3.15 est.) — highest subtype accuracy in the sweep to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>meta-llama-llama-3.3-70b-instruct_sorter_v13_subtype_langfuse</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>509</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-3.3-70b-instruct</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>v13</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.9941</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.8782</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>0.8998</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>0.9424</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>509</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>0.8487</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>0.9056999999999999</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>0.0285</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>0.9862</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="U9" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="V9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="W9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X9" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Y9" s="6" t="n">
+        <v>0.9231</v>
+      </c>
+      <c r="Z9" s="6" t="n">
+        <v>0.9545</v>
+      </c>
+      <c r="AA9" s="6" t="n">
+        <v>0.6923</v>
+      </c>
+      <c r="AB9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC9" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AD9" s="6" t="n">
+        <v>0.9688</v>
+      </c>
+      <c r="AE9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF9" s="6" t="n">
+        <v>0.8667</v>
+      </c>
+      <c r="AG9" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AH9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ9" s="6" t="n">
+        <v>0.9091</v>
+      </c>
+      <c r="AK9" s="6" t="n">
+        <v>0.8235</v>
+      </c>
+      <c r="AL9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM9" s="6" t="n">
+        <v>0.6471</v>
+      </c>
+      <c r="AN9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO9" s="6" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="AP9" s="6" t="n">
+        <v>0.6667</v>
+      </c>
+      <c r="AQ9" s="6" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="AR9" s="6" t="n">
+        <v>0.8214</v>
+      </c>
+      <c r="AS9" s="6" t="n">
+        <v>0.9677</v>
+      </c>
+      <c r="AT9" s="6" t="n">
+        <v>0.9688</v>
+      </c>
+      <c r="AU9" s="6" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="AV9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW9" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AX9" s="6" t="n">
+        <v>0.9231</v>
+      </c>
+      <c r="AY9" s="6" t="n">
+        <v>0.9545</v>
+      </c>
+      <c r="AZ9" s="6" t="n">
+        <v>0.6923</v>
+      </c>
+      <c r="BA9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB9" s="6" t="n">
+        <v>0.8571</v>
+      </c>
+      <c r="BC9" s="6" t="n">
+        <v>0.9688</v>
+      </c>
+      <c r="BD9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE9" s="6" t="n">
+        <v>0.8667</v>
+      </c>
+      <c r="BF9" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BG9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI9" s="6" t="n">
+        <v>0.9394</v>
+      </c>
+      <c r="BJ9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL9" s="6" t="n">
+        <v>0.6471</v>
+      </c>
+      <c r="BM9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN9" s="6" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="BO9" s="6" t="n">
+        <v>0.6667</v>
+      </c>
+      <c r="BP9" s="6" t="n">
+        <v>0.9167</v>
+      </c>
+      <c r="BQ9" s="6" t="n">
+        <v>0.8214</v>
+      </c>
+      <c r="BR9" s="6" t="n">
+        <v>0.9677</v>
+      </c>
+      <c r="BS9" s="6" t="n">
+        <v>0.9688</v>
+      </c>
+      <c r="BT9" s="6" t="n">
+        <v>0.8889</v>
+      </c>
+      <c r="BU9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="BW9" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="BX9" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="BY9" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="BZ9" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="CA9" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="CB9" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="CC9" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="CD9" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="CE9" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="CF9" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="CG9" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="CH9" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="CI9" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="CJ9" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="CK9" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="CL9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CM9" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="CN9" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="CO9" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="CP9" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="CQ9" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="CR9" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="CS9" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="CT9" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="CU9" s="4" t="n">
+        <v>6584627</v>
+      </c>
+      <c r="CV9" s="4" t="n">
+        <v>73143</v>
+      </c>
+      <c r="CW9" s="4" t="n">
+        <v>6657770</v>
+      </c>
+      <c r="CX9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ9" s="3" t="n"/>
+      <c r="DA9" s="4" t="n">
+        <v>509</v>
+      </c>
+      <c r="DB9" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="DC9" s="4" t="n">
+        <v>4096</v>
+      </c>
+      <c r="DD9" s="4" t="n">
+        <v>100000</v>
+      </c>
+      <c r="DE9" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="DF9" s="3" t="inlineStr">
+        <is>
+          <t>llm-mailroom/mailroom-cuad-contracts-full</t>
+        </is>
+      </c>
+      <c r="DG9" s="4" t="n">
+        <v>509</v>
+      </c>
+      <c r="DH9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="DI9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ9" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="DK9" s="3" t="inlineStr">
+        <is>
+          <t>Full-509 benchmark (KANBAN-042) — llama 3.3 70B instruct arm (OpenRouter-billed, no local price)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:DK7"/>
+  <autoFilter ref="A1:DK9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>